<commit_message>
Add Diagnostics for Missed Forecasts; jupyter tools for extracting data from HTML, logs, and API
</commit_message>
<xml_diff>
--- a/conversation and context docs/forecasting_bot_improvement_ideas_edit 02-08-2026.xlsx
+++ b/conversation and context docs/forecasting_bot_improvement_ideas_edit 02-08-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Donni\projects\metac_bot_Spring_2026\conversation and context docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB87C3B-AA80-4B09-94CD-E44A269D6CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A3F46B-CBB0-4201-B62E-66613E43460D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28410" yWindow="-2310" windowWidth="16240" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10580" yWindow="0" windowWidth="15110" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -49,12 +49,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="H45" authorId="0" shapeId="0" xr:uid="{0216EDEE-A194-4DFF-824A-1093C1A364CA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Donni:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1 to 10</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="79">
   <si>
     <t>Date</t>
   </si>
@@ -281,13 +305,16 @@
     <t>done (6 runs)</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>Scoring Understanding</t>
   </si>
   <si>
     <t>Orig Order</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>unclear</t>
   </si>
 </sst>
 </file>
@@ -344,7 +371,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -367,13 +394,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -687,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -696,7 +737,7 @@
     <col min="4" max="4" width="71.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -713,10 +754,13 @@
         <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -729,14 +773,14 @@
       <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="E2" t="s">
-        <v>74</v>
-      </c>
       <c r="F2">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -749,14 +793,14 @@
       <c r="D3" t="s">
         <v>35</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
         <v>72</v>
       </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -769,14 +813,14 @@
       <c r="D4" t="s">
         <v>36</v>
       </c>
-      <c r="E4" t="s">
-        <v>72</v>
-      </c>
       <c r="F4">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -789,14 +833,14 @@
       <c r="D5" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
-        <v>72</v>
-      </c>
       <c r="F5">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -809,14 +853,14 @@
       <c r="D6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" t="s">
-        <v>72</v>
-      </c>
       <c r="F6">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -829,14 +873,14 @@
       <c r="D7" t="s">
         <v>46</v>
       </c>
-      <c r="E7" t="s">
-        <v>72</v>
-      </c>
       <c r="F7">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -849,14 +893,14 @@
       <c r="D8" t="s">
         <v>47</v>
       </c>
-      <c r="E8" t="s">
-        <v>72</v>
-      </c>
       <c r="F8">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -869,14 +913,14 @@
       <c r="D9" t="s">
         <v>49</v>
       </c>
-      <c r="E9" t="s">
-        <v>72</v>
-      </c>
       <c r="F9">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -889,19 +933,19 @@
       <c r="D10" t="s">
         <v>51</v>
       </c>
-      <c r="E10" t="s">
-        <v>75</v>
-      </c>
       <c r="F10">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
         <v>26</v>
@@ -909,14 +953,14 @@
       <c r="D11" t="s">
         <v>60</v>
       </c>
-      <c r="E11" t="s">
-        <v>75</v>
+      <c r="E11">
+        <v>5</v>
       </c>
       <c r="F11">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -926,7 +970,7 @@
       <c r="C12" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E12">
@@ -935,8 +979,11 @@
       <c r="F12">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -946,7 +993,7 @@
       <c r="C13" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>65</v>
       </c>
       <c r="E13">
@@ -956,7 +1003,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -966,7 +1013,7 @@
       <c r="C14" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E14">
@@ -976,7 +1023,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -996,7 +1043,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1046,7 +1093,7 @@
       <c r="C18" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E18">
@@ -1104,7 +1151,7 @@
         <v>22</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D21" t="s">
         <v>55</v>
@@ -1336,7 +1383,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1356,7 +1403,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -1376,7 +1423,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>5</v>
       </c>
@@ -1396,7 +1443,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -1416,7 +1463,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>18</v>
       </c>
@@ -1436,7 +1483,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1456,7 +1503,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -1476,7 +1523,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -1496,7 +1543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -1513,7 +1560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -1527,6 +1574,846 @@
         <v>44</v>
       </c>
       <c r="F42">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D45" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D46" t="s">
+        <v>14</v>
+      </c>
+      <c r="E46" t="s">
+        <v>22</v>
+      </c>
+      <c r="F46" t="s">
+        <v>24</v>
+      </c>
+      <c r="G46" t="s">
+        <v>50</v>
+      </c>
+      <c r="I46">
+        <v>20</v>
+      </c>
+      <c r="J46" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D47" t="s">
+        <v>6</v>
+      </c>
+      <c r="E47" t="s">
+        <v>22</v>
+      </c>
+      <c r="F47" t="s">
+        <v>23</v>
+      </c>
+      <c r="G47" t="s">
+        <v>35</v>
+      </c>
+      <c r="I47">
+        <v>5</v>
+      </c>
+      <c r="J47" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D48" t="s">
+        <v>6</v>
+      </c>
+      <c r="E48" t="s">
+        <v>21</v>
+      </c>
+      <c r="F48" t="s">
+        <v>23</v>
+      </c>
+      <c r="G48" t="s">
+        <v>36</v>
+      </c>
+      <c r="I48">
+        <v>6</v>
+      </c>
+      <c r="J48" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>22</v>
+      </c>
+      <c r="F49" t="s">
+        <v>23</v>
+      </c>
+      <c r="G49" t="s">
+        <v>38</v>
+      </c>
+      <c r="I49">
+        <v>8</v>
+      </c>
+      <c r="J49" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="50" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50" t="s">
+        <v>22</v>
+      </c>
+      <c r="F50" t="s">
+        <v>23</v>
+      </c>
+      <c r="G50" t="s">
+        <v>39</v>
+      </c>
+      <c r="I50">
+        <v>9</v>
+      </c>
+      <c r="J50" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="51" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" t="s">
+        <v>22</v>
+      </c>
+      <c r="F51" t="s">
+        <v>24</v>
+      </c>
+      <c r="G51" t="s">
+        <v>46</v>
+      </c>
+      <c r="I51">
+        <v>16</v>
+      </c>
+      <c r="J51" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" t="s">
+        <v>22</v>
+      </c>
+      <c r="F52" t="s">
+        <v>24</v>
+      </c>
+      <c r="G52" t="s">
+        <v>47</v>
+      </c>
+      <c r="I52">
+        <v>17</v>
+      </c>
+      <c r="J52" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="53" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" t="s">
+        <v>22</v>
+      </c>
+      <c r="F53" t="s">
+        <v>24</v>
+      </c>
+      <c r="G53" t="s">
+        <v>49</v>
+      </c>
+      <c r="I53">
+        <v>19</v>
+      </c>
+      <c r="J53" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="54" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D54" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54" t="s">
+        <v>22</v>
+      </c>
+      <c r="F54" t="s">
+        <v>24</v>
+      </c>
+      <c r="G54" t="s">
+        <v>51</v>
+      </c>
+      <c r="I54">
+        <v>21</v>
+      </c>
+      <c r="J54" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D55" t="s">
+        <v>16</v>
+      </c>
+      <c r="E55" t="s">
+        <v>22</v>
+      </c>
+      <c r="F55" t="s">
+        <v>26</v>
+      </c>
+      <c r="G55" t="s">
+        <v>60</v>
+      </c>
+      <c r="H55">
+        <v>5</v>
+      </c>
+      <c r="I55">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="56" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D56" t="s">
+        <v>17</v>
+      </c>
+      <c r="E56" t="s">
+        <v>22</v>
+      </c>
+      <c r="F56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H56">
+        <v>10</v>
+      </c>
+      <c r="I56">
+        <v>31</v>
+      </c>
+      <c r="J56" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="57" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D57" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" t="s">
+        <v>22</v>
+      </c>
+      <c r="F57" t="s">
+        <v>27</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H57">
+        <v>9</v>
+      </c>
+      <c r="I57">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D58" t="s">
+        <v>15</v>
+      </c>
+      <c r="E58" t="s">
+        <v>22</v>
+      </c>
+      <c r="F58" t="s">
+        <v>26</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H58">
+        <v>8</v>
+      </c>
+      <c r="I58">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D59" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" t="s">
+        <v>22</v>
+      </c>
+      <c r="F59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G59" t="s">
+        <v>63</v>
+      </c>
+      <c r="H59">
+        <v>8</v>
+      </c>
+      <c r="I59">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D60" t="s">
+        <v>4</v>
+      </c>
+      <c r="E60" t="s">
+        <v>22</v>
+      </c>
+      <c r="F60" t="s">
+        <v>28</v>
+      </c>
+      <c r="G60" t="s">
+        <v>66</v>
+      </c>
+      <c r="H60">
+        <v>8</v>
+      </c>
+      <c r="I60">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="61" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D61" t="s">
+        <v>18</v>
+      </c>
+      <c r="E61" t="s">
+        <v>22</v>
+      </c>
+      <c r="F61" t="s">
+        <v>29</v>
+      </c>
+      <c r="G61" t="s">
+        <v>68</v>
+      </c>
+      <c r="H61">
+        <v>8</v>
+      </c>
+      <c r="I61">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="62" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D62" t="s">
+        <v>20</v>
+      </c>
+      <c r="E62" t="s">
+        <v>22</v>
+      </c>
+      <c r="F62" t="s">
+        <v>29</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H62">
+        <v>8</v>
+      </c>
+      <c r="I62">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="63" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D63" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" t="s">
+        <v>22</v>
+      </c>
+      <c r="F63" t="s">
+        <v>23</v>
+      </c>
+      <c r="G63" t="s">
+        <v>40</v>
+      </c>
+      <c r="H63">
+        <v>7</v>
+      </c>
+      <c r="I63">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="4:10" x14ac:dyDescent="0.35">
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>22</v>
+      </c>
+      <c r="F64" t="s">
+        <v>23</v>
+      </c>
+      <c r="G64" t="s">
+        <v>41</v>
+      </c>
+      <c r="H64">
+        <v>7</v>
+      </c>
+      <c r="I64">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>22</v>
+      </c>
+      <c r="F65" t="s">
+        <v>75</v>
+      </c>
+      <c r="G65" t="s">
+        <v>55</v>
+      </c>
+      <c r="H65">
+        <v>7</v>
+      </c>
+      <c r="I65">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="66" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D66" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" t="s">
+        <v>22</v>
+      </c>
+      <c r="F66" t="s">
+        <v>27</v>
+      </c>
+      <c r="G66" t="s">
+        <v>62</v>
+      </c>
+      <c r="H66">
+        <v>7</v>
+      </c>
+      <c r="I66">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D67" t="s">
+        <v>19</v>
+      </c>
+      <c r="E67" t="s">
+        <v>22</v>
+      </c>
+      <c r="F67" t="s">
+        <v>28</v>
+      </c>
+      <c r="G67" t="s">
+        <v>67</v>
+      </c>
+      <c r="H67">
+        <v>7</v>
+      </c>
+      <c r="I67">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="68" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D68" t="s">
+        <v>4</v>
+      </c>
+      <c r="E68" t="s">
+        <v>22</v>
+      </c>
+      <c r="F68" t="s">
+        <v>30</v>
+      </c>
+      <c r="G68" t="s">
+        <v>70</v>
+      </c>
+      <c r="H68">
+        <v>7</v>
+      </c>
+      <c r="I68">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="69" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D69" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" t="s">
+        <v>22</v>
+      </c>
+      <c r="F69" t="s">
+        <v>24</v>
+      </c>
+      <c r="G69" t="s">
+        <v>52</v>
+      </c>
+      <c r="H69">
+        <v>6</v>
+      </c>
+      <c r="I69">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>22</v>
+      </c>
+      <c r="F70" t="s">
+        <v>30</v>
+      </c>
+      <c r="G70" t="s">
+        <v>71</v>
+      </c>
+      <c r="H70">
+        <v>6</v>
+      </c>
+      <c r="I70">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="71" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D71" t="s">
+        <v>4</v>
+      </c>
+      <c r="E71" t="s">
+        <v>22</v>
+      </c>
+      <c r="F71" t="s">
+        <v>23</v>
+      </c>
+      <c r="G71" t="s">
+        <v>32</v>
+      </c>
+      <c r="H71">
+        <v>5</v>
+      </c>
+      <c r="I71">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D72" t="s">
+        <v>7</v>
+      </c>
+      <c r="E72" t="s">
+        <v>22</v>
+      </c>
+      <c r="F72" t="s">
+        <v>23</v>
+      </c>
+      <c r="G72" t="s">
+        <v>37</v>
+      </c>
+      <c r="H72">
+        <v>5</v>
+      </c>
+      <c r="I72">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D73" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" t="s">
+        <v>22</v>
+      </c>
+      <c r="F73" t="s">
+        <v>23</v>
+      </c>
+      <c r="G73" t="s">
+        <v>42</v>
+      </c>
+      <c r="H73">
+        <v>5</v>
+      </c>
+      <c r="I73">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="74" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D74" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>22</v>
+      </c>
+      <c r="F74" t="s">
+        <v>23</v>
+      </c>
+      <c r="G74" t="s">
+        <v>43</v>
+      </c>
+      <c r="H74">
+        <v>5</v>
+      </c>
+      <c r="I74">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="75" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D75" t="s">
+        <v>5</v>
+      </c>
+      <c r="E75" t="s">
+        <v>22</v>
+      </c>
+      <c r="F75" t="s">
+        <v>24</v>
+      </c>
+      <c r="G75" t="s">
+        <v>45</v>
+      </c>
+      <c r="H75">
+        <v>5</v>
+      </c>
+      <c r="I75">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D76" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s">
+        <v>22</v>
+      </c>
+      <c r="F76" t="s">
+        <v>25</v>
+      </c>
+      <c r="G76" t="s">
+        <v>53</v>
+      </c>
+      <c r="H76">
+        <v>5</v>
+      </c>
+      <c r="I76">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="77" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D77" t="s">
+        <v>11</v>
+      </c>
+      <c r="E77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F77" t="s">
+        <v>25</v>
+      </c>
+      <c r="G77" t="s">
+        <v>54</v>
+      </c>
+      <c r="H77">
+        <v>5</v>
+      </c>
+      <c r="I77">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D78" t="s">
+        <v>12</v>
+      </c>
+      <c r="E78" t="s">
+        <v>22</v>
+      </c>
+      <c r="F78" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" t="s">
+        <v>57</v>
+      </c>
+      <c r="H78">
+        <v>5</v>
+      </c>
+      <c r="I78">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="79" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D79" t="s">
+        <v>5</v>
+      </c>
+      <c r="E79" t="s">
+        <v>22</v>
+      </c>
+      <c r="F79" t="s">
+        <v>23</v>
+      </c>
+      <c r="G79" t="s">
+        <v>33</v>
+      </c>
+      <c r="H79">
+        <v>4</v>
+      </c>
+      <c r="I79">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D80" t="s">
+        <v>12</v>
+      </c>
+      <c r="E80" t="s">
+        <v>21</v>
+      </c>
+      <c r="F80" t="s">
+        <v>26</v>
+      </c>
+      <c r="G80" t="s">
+        <v>56</v>
+      </c>
+      <c r="H80">
+        <v>4</v>
+      </c>
+      <c r="I80">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D81" t="s">
+        <v>18</v>
+      </c>
+      <c r="E81" t="s">
+        <v>22</v>
+      </c>
+      <c r="F81" t="s">
+        <v>27</v>
+      </c>
+      <c r="G81" t="s">
+        <v>64</v>
+      </c>
+      <c r="H81">
+        <v>4</v>
+      </c>
+      <c r="I81">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="82" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D82" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" t="s">
+        <v>22</v>
+      </c>
+      <c r="F82" t="s">
+        <v>24</v>
+      </c>
+      <c r="G82" t="s">
+        <v>48</v>
+      </c>
+      <c r="H82">
+        <v>3</v>
+      </c>
+      <c r="I82">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="83" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D83" t="s">
+        <v>12</v>
+      </c>
+      <c r="E83" t="s">
+        <v>22</v>
+      </c>
+      <c r="F83" t="s">
+        <v>26</v>
+      </c>
+      <c r="G83" t="s">
+        <v>58</v>
+      </c>
+      <c r="H83">
+        <v>3</v>
+      </c>
+      <c r="I83">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="84" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D84" t="s">
+        <v>5</v>
+      </c>
+      <c r="E84" t="s">
+        <v>22</v>
+      </c>
+      <c r="F84" t="s">
+        <v>23</v>
+      </c>
+      <c r="G84" t="s">
+        <v>34</v>
+      </c>
+      <c r="H84">
+        <v>2</v>
+      </c>
+      <c r="I84">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D85" t="s">
+        <v>4</v>
+      </c>
+      <c r="E85" t="s">
+        <v>21</v>
+      </c>
+      <c r="F85" t="s">
+        <v>23</v>
+      </c>
+      <c r="G85" t="s">
+        <v>31</v>
+      </c>
+      <c r="I85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E86" t="s">
+        <v>21</v>
+      </c>
+      <c r="F86" t="s">
+        <v>24</v>
+      </c>
+      <c r="G86" t="s">
+        <v>44</v>
+      </c>
+      <c r="I86">
         <v>14</v>
       </c>
     </row>
@@ -1535,6 +2422,7 @@
     <sortCondition descending="1" ref="E2:E42"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>